<commit_message>
Validate AbDev-Lite v0.6 candidate prioritization
</commit_message>
<xml_diff>
--- a/outputs/abdev_lite_results.xlsx
+++ b/outputs/abdev_lite_results.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input_Cleaned" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sequence_QC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chain_Properties" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numbering_Residues" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Region_Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liability_Sites" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liability_Region_Map" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chain_Risk_Scores" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Humanness_Results" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Antibody_Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Input_Cleaned" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sequence_QC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chain_Properties" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Numbering_Residues" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Region_Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Liability_Sites" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Liability_Region_Map" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Chain_Risk_Scores" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Humanness_Results" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Antibody_Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Candidate_Ranking" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1912,6 +1913,492 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>antibody_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>molecule_format</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>number_of_chains</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>total_risk_score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cdr_adjusted_total_risk_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>max_chain_risk_class</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>cdr_adjusted_max_risk_class</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>total_cdr_liabilities</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>total_fr_liabilities</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>max_humanness_risk_class</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>high_humanness_risk_chain_count</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>non_human_like_chain_count</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>combined_developability_humanness_flag</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>final_priority_score</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>final_priority_class</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>decision_label</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>review_reason</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>next_step_recommendation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ab001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>mAb</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Developability review recommended</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Deprioritize or redesign before progression</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BadSeq001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mAb</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Developability review recommended</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Deprioritize or redesign before progression</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BsAb001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BsAb</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>High priority engineering review</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Deprioritize or redesign before progression</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>High humanness risk based on imported assessment; High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Full001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mAb</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Developability review recommended</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Deprioritize or redesign before progression</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>High CDR-adjusted developability burden</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VHH001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>VHH</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>High priority engineering review</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Deprioritize or redesign before progression</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>High humanness risk based on imported assessment; High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3651,7 +4138,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3722,7 +4209,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -3793,7 +4280,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -3864,7 +4351,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -3935,7 +4422,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -4006,7 +4493,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -4077,7 +4564,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -4148,7 +4635,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
+          <t>IMGT numbering failed: No module named 'anarci'</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">

</xml_diff>

<commit_message>
Release AbDev-Lite v0.7 with Expreso-lite formulation integration
</commit_message>
<xml_diff>
--- a/outputs/abdev_lite_results.xlsx
+++ b/outputs/abdev_lite_results.xlsx
@@ -18,6 +18,9 @@
     <sheet name="Humanness_Results" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Antibody_Summary" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Candidate_Ranking" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Formulation_Features" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Expreso_Predictions" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Formulation_Recommendations" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2399,6 +2402,1564 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AH6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>antibody_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>molecule_format</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>number_of_chains</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>average_sequence_length</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>total_sequence_length</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>average_theoretical_pI</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>max_theoretical_pI</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>min_theoretical_pI</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>average_gravy</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>max_gravy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>average_instability_index</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>total_cysteine_count</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>total_methionine_count</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>total_tryptophan_count</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>total_asparagine_count</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>total_aspartic_acid_count</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>total_lysine_count</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>total_arginine_count</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>hydrophobic_residue_fraction_mean</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>aromatic_residue_fraction_mean</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>positive_residue_fraction_mean</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>negative_residue_fraction_mean</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>total_risk_score</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>cdr_adjusted_total_risk_score</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>total_cdr_liabilities</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>total_fr_liabilities</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>total_nglycosylation_motifs</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>total_deamidation_motifs</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>total_isomerization_motifs</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>total_oxidation_motifs</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>total_hydrophobic_patch_proxy</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>max_humanness_risk_class</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>final_priority_class</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>final_priority_score</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ab001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>mAb</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>221</v>
+      </c>
+      <c r="F2" t="n">
+        <v>8.541499999999999</v>
+      </c>
+      <c r="G2" t="n">
+        <v>9.036</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8.047000000000001</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.2948</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-0.1877</v>
+      </c>
+      <c r="K2" t="n">
+        <v>40.473</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>6</v>
+      </c>
+      <c r="P2" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>8</v>
+      </c>
+      <c r="R2" t="n">
+        <v>11</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.3702</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.1084</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.0862</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.0678</v>
+      </c>
+      <c r="W2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="X2" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>9</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BadSeq001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mAb</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>22</v>
+      </c>
+      <c r="E3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.2818</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.2818</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-0.773</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>5</v>
+      </c>
+      <c r="N3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O3" t="n">
+        <v>2</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.7272999999999999</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.2273</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.0455</v>
+      </c>
+      <c r="W3" t="n">
+        <v>21</v>
+      </c>
+      <c r="X3" t="n">
+        <v>21</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AH3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BsAb001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BsAb</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>111.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>446</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7.5555</v>
+      </c>
+      <c r="G4" t="n">
+        <v>8.981</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.337</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.3484</v>
+      </c>
+      <c r="J4" t="n">
+        <v>-0.2453</v>
+      </c>
+      <c r="K4" t="n">
+        <v>39.9902</v>
+      </c>
+      <c r="L4" t="n">
+        <v>8</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N4" t="n">
+        <v>14</v>
+      </c>
+      <c r="O4" t="n">
+        <v>16</v>
+      </c>
+      <c r="P4" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>15</v>
+      </c>
+      <c r="R4" t="n">
+        <v>23</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.3825</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.1252</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.08740000000000001</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.07630000000000001</v>
+      </c>
+      <c r="W4" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="X4" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>19</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>8</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AH4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Full001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>mAb</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>227</v>
+      </c>
+      <c r="E5" t="n">
+        <v>227</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8.808999999999999</v>
+      </c>
+      <c r="G5" t="n">
+        <v>8.808999999999999</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8.808999999999999</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.1692</v>
+      </c>
+      <c r="J5" t="n">
+        <v>-0.1692</v>
+      </c>
+      <c r="K5" t="n">
+        <v>45.005</v>
+      </c>
+      <c r="L5" t="n">
+        <v>7</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>4</v>
+      </c>
+      <c r="O5" t="n">
+        <v>8</v>
+      </c>
+      <c r="P5" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>12</v>
+      </c>
+      <c r="R5" t="n">
+        <v>6</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.0881</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.0925</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.0573</v>
+      </c>
+      <c r="W5" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="X5" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>7</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VHH001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>VHH</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>115</v>
+      </c>
+      <c r="E6" t="n">
+        <v>115</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8.638999999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8.638999999999999</v>
+      </c>
+      <c r="H6" t="n">
+        <v>8.638999999999999</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-0.2504</v>
+      </c>
+      <c r="J6" t="n">
+        <v>-0.2504</v>
+      </c>
+      <c r="K6" t="n">
+        <v>31.669</v>
+      </c>
+      <c r="L6" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>4</v>
+      </c>
+      <c r="R6" t="n">
+        <v>6</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.4087</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.1217</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.0696</v>
+      </c>
+      <c r="W6" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="X6" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>antibody_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>model_available</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>model_status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>prediction_mode</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>recommended_buffer_ph_modifier_probability</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sugar_stabilizer_probability</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>polyol_stabilizer_probability</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>surfactant_probability</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>amino_acid_stabilizer_probability</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>antioxidant_probability</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>chelating_agent_probability</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>salt_ionic_strength_modifier_probability</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>preservative_probability</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>expreso_prediction_warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ab001</t>
+        </is>
+      </c>
+      <c r="B2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>model_not_found</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>rule_based_fallback</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Expreso-lite model files were not found. Rule-based fallback recommendation was used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BadSeq001</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>model_not_found</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>rule_based_fallback</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Expreso-lite model files were not found. Rule-based fallback recommendation was used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BsAb001</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>model_not_found</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>rule_based_fallback</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Expreso-lite model files were not found. Rule-based fallback recommendation was used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Full001</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>model_not_found</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>rule_based_fallback</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Expreso-lite model files were not found. Rule-based fallback recommendation was used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VHH001</t>
+        </is>
+      </c>
+      <c r="B6" t="b">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>model_not_found</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>rule_based_fallback</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Expreso-lite model files were not found. Rule-based fallback recommendation was used.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>antibody_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>formulation_risk_class</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>formulation_risk_score</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>recommended_excipient_classes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>top_excipient_class_1</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>top_excipient_class_2</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>top_excipient_class_3</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>buffer_ph_direction</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>surfactant_consideration</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sugar_polyol_consideration</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>oxidation_control_consideration</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ionic_strength_consideration</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>formulation_review_reason</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>formulation_next_step_recommendation</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>formulation_disclaimer</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ab001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>sugar stabilizer; antioxidant; surfactant</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>sugar stabilizer</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>antioxidant</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>surfactant</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Include broad buffer and pH screening; review pH-sensitive motifs</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Prioritize surfactant screening due to hydrophobicity signal</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Prioritize sugar/polyol stabilizer screening due to instability signal</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Consider antioxidant and oxidation-control review</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Optional ionic strength screen</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Elevated oxidation-prone residue count; Hydrophobicity or hydrophobic patch proxy suggests surfactant review; High CDR-adjusted developability burden; Instability index suggests stabilizer screening; Deamidation/isomerization motif burden suggests pH sensitivity review</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Prioritize preformulation risk review before scale-up or advanced developability studies</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Formulation recommendations are computational triage outputs based on sequence-level features and optional Expreso-lite model predictions. They are intended to support early preformulation planning only and do not replace experimental formulation screening, stability studies, or CMC evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BadSeq001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>13</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>surfactant; buffer / pH modifier; antioxidant</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>surfactant</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>buffer / pH modifier</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>antioxidant</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Prioritize pH screening above the low theoretical pI range; review pH-sensitive motifs</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Prioritize surfactant screening due to hydrophobicity signal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Consider sugar stabilizer as a default early screen</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Consider antioxidant and oxidation-control review</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Include ionic strength screen because theoretical pI is shifted</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Elevated oxidation-prone residue count; Hydrophobicity or hydrophobic patch proxy suggests surfactant review; High CDR-adjusted developability burden; Theoretical pI is outside the broad neutral range; Deamidation/isomerization motif burden suggests pH sensitivity review</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Prioritize preformulation risk review before scale-up or advanced developability studies</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Formulation recommendations are computational triage outputs based on sequence-level features and optional Expreso-lite model predictions. They are intended to support early preformulation planning only and do not replace experimental formulation screening, stability studies, or CMC evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BsAb001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>antioxidant; surfactant; buffer / pH modifier</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>antioxidant</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>surfactant</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>buffer / pH modifier</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Include broad buffer and pH screening; review pH-sensitive motifs</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Prioritize surfactant screening due to hydrophobicity signal</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Consider sugar stabilizer as a default early screen</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Consider antioxidant and oxidation-control review</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Optional ionic strength screen</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Elevated oxidation-prone residue count; Hydrophobicity or hydrophobic patch proxy suggests surfactant review; High CDR-adjusted developability burden; Deamidation/isomerization motif burden suggests pH sensitivity review</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Prioritize preformulation risk review before scale-up or advanced developability studies</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Formulation recommendations are computational triage outputs based on sequence-level features and optional Expreso-lite model predictions. They are intended to support early preformulation planning only and do not replace experimental formulation screening, stability studies, or CMC evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Full001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>sugar stabilizer; antioxidant; surfactant</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>sugar stabilizer</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>antioxidant</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>surfactant</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Include broad buffer and pH screening; review pH-sensitive motifs</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Prioritize surfactant screening due to hydrophobicity signal</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Prioritize sugar/polyol stabilizer screening due to instability signal</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Consider antioxidant and oxidation-control review</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Optional ionic strength screen</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Elevated oxidation-prone residue count; Hydrophobicity or hydrophobic patch proxy suggests surfactant review; High CDR-adjusted developability burden; Instability index suggests stabilizer screening; Deamidation/isomerization motif burden suggests pH sensitivity review; Cysteine count suggests redox-related review</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Prioritize preformulation risk review before scale-up or advanced developability studies</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Formulation recommendations are computational triage outputs based on sequence-level features and optional Expreso-lite model predictions. They are intended to support early preformulation planning only and do not replace experimental formulation screening, stability studies, or CMC evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VHH001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>antioxidant; surfactant; buffer / pH modifier</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>antioxidant</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>surfactant</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>buffer / pH modifier</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Include broad buffer and pH screening; review pH-sensitive motifs</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Prioritize surfactant screening due to hydrophobicity signal</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Consider sugar stabilizer as a default early screen</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Consider antioxidant and oxidation-control review</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Optional ionic strength screen</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Elevated oxidation-prone residue count; Hydrophobicity or hydrophobic patch proxy suggests surfactant review; High CDR-adjusted developability burden; Deamidation/isomerization motif burden suggests pH sensitivity review</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Prioritize preformulation risk review before scale-up or advanced developability studies</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Formulation recommendations are computational triage outputs based on sequence-level features and optional Expreso-lite model predictions. They are intended to support early preformulation planning only and do not replace experimental formulation screening, stability studies, or CMC evaluation.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Release AbDev-Lite v0.8 with structure result import
</commit_message>
<xml_diff>
--- a/outputs/abdev_lite_results.xlsx
+++ b/outputs/abdev_lite_results.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Input_Cleaned" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sequence_QC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chain_Properties" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Numbering_Residues" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Region_Summary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Liability_Sites" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Liability_Region_Map" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Chain_Risk_Scores" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Humanness_Results" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Antibody_Summary" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Candidate_Ranking" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Formulation_Features" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Expreso_Predictions" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Formulation_Recommendations" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Input_Cleaned" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sequence_QC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chain_Properties" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numbering_Residues" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Region_Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liability_Sites" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liability_Region_Map" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chain_Risk_Scores" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Humanness_Results" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Antibody_Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate_Ranking" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulation_Features" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expreso_Predictions" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulation_Recommendations" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure_Results" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structural_Risk_Summary" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1106,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF6"/>
+  <dimension ref="A1:AK6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1270,6 +1272,31 @@
           <t>combined_developability_humanness_flag</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>structure_available</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>structural_risk_class</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>structural_risk_score</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>structural_review_reason</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>structural_next_step_recommendation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1355,7 +1382,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Input sequences passed basic QC; No obvious N-glycosylation motif detected in variable region; No obvious unpaired cysteine proxy detected; No obvious liability motif mapped to CDR regions by IMGT-based computational assignment; Human-likeness metrics suggest low humanness risk based on imported assessment</t>
+          <t>Input sequences passed basic QC; No obvious N-glycosylation motif detected in variable region; No obvious unpaired cysteine proxy detected; No obvious liability motif mapped to CDR regions by IMGT-based computational assignment; Human-likeness metrics suggest low humanness risk based on imported assessment; Imported structure metrics suggest low structural risk in this MVP assessment</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -1400,6 +1427,27 @@
       <c r="AF2" t="inlineStr">
         <is>
           <t>Developability review recommended</t>
+        </is>
+      </c>
+      <c r="AG2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>No major structural risk flag detected from imported metrics</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Imported structure metrics do not indicate a major structural review flag in this MVP assessment</t>
         </is>
       </c>
     </row>
@@ -1526,6 +1574,27 @@
           <t>Developability review recommended</t>
         </is>
       </c>
+      <c r="AG3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="AI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>No external structure prediction result was provided</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Import external structure prediction summary metrics if structural triage is needed</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1656,6 +1725,27 @@
       <c r="AF4" t="inlineStr">
         <is>
           <t>High priority engineering review</t>
+        </is>
+      </c>
+      <c r="AG4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AI4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>No major structural risk flag detected from imported metrics</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Review imported structure confidence and patch annotations before progression</t>
         </is>
       </c>
     </row>
@@ -1782,6 +1872,27 @@
           <t>Developability review recommended</t>
         </is>
       </c>
+      <c r="AG5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="AI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>No external structure prediction result was provided</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Import external structure prediction summary metrics if structural triage is needed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1908,6 +2019,27 @@
       <c r="AF6" t="inlineStr">
         <is>
           <t>High priority engineering review</t>
+        </is>
+      </c>
+      <c r="AG6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>No external structure prediction result was provided</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>Import external structure prediction summary metrics if structural triage is needed</t>
         </is>
       </c>
     </row>
@@ -1922,7 +2054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1993,25 +2125,40 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>structure_available</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>structural_risk_class</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>structural_risk_score</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>final_priority_score</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>final_priority_class</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>decision_label</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>review_reason</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>next_step_recommendation</t>
         </is>
@@ -2069,25 +2216,36 @@
           <t>Developability review recommended</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Deprioritize or redesign before progression</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
         </is>
@@ -2145,25 +2303,36 @@
           <t>Developability review recommended</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="N3" t="b">
         <v>0</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Deprioritize or redesign before progression</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>High CDR-adjusted developability burden; No structure result imported; Sequence-level hydrophobic patch proxy detected</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
         </is>
@@ -2221,25 +2390,36 @@
           <t>High priority engineering review</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q4" t="n">
         <v>0</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Deprioritize or redesign before progression</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>High humanness risk based on imported assessment; High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
         </is>
@@ -2297,25 +2477,36 @@
           <t>Developability review recommended</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" t="b">
         <v>0</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Deprioritize or redesign before progression</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>High CDR-adjusted developability burden</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>High CDR-adjusted developability burden; No structure result imported</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
         <is>
           <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
         </is>
@@ -2373,25 +2564,36 @@
           <t>High priority engineering review</t>
         </is>
       </c>
-      <c r="N6" t="n">
+      <c r="N6" t="b">
         <v>0</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Deprioritize or redesign before progression</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>High humanness risk based on imported assessment; High CDR-adjusted developability burden; Sequence-level hydrophobic patch proxy detected</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>High humanness risk based on imported assessment; High CDR-adjusted developability burden; No structure result imported; Sequence-level hydrophobic patch proxy detected</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
         <is>
           <t>Consider redesign, deprioritization, or additional humanization/developability review</t>
         </is>
@@ -3960,6 +4162,854 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>antibody_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sequence_scope</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>structure_tool</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>structure_model_file</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>structure_status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>mean_plddt</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cdr1_plddt</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>cdr2_plddt</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>cdr3_plddt</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>vh_vl_orientation_confidence</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>predicted_surface_hydrophobic_patch_score</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>predicted_aggregation_patch_score</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>predicted_charge_patch_score</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>structural_notes</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>merge_status</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>merge_warning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ab001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>VHVL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>VH,VL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IgFold</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Ab001_VHVL.pdb</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>86</v>
+      </c>
+      <c r="I2" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>82</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Low structural risk example</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>matched_by_antibody_id</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BsAb001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ArmA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BsAb001_ArmA_model.pdb</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>76</v>
+      </c>
+      <c r="H3" t="n">
+        <v>74</v>
+      </c>
+      <c r="I3" t="n">
+        <v>72</v>
+      </c>
+      <c r="J3" t="n">
+        <v>71</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Medium structural risk example from orientation warning</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>matched_by_antibody_id</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ab_CDR3Low</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>IgFold</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Ab_CDR3Low_VH.pdb</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>78</v>
+      </c>
+      <c r="H4" t="n">
+        <v>75</v>
+      </c>
+      <c r="I4" t="n">
+        <v>73</v>
+      </c>
+      <c r="J4" t="n">
+        <v>55</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Low CDR3 pLDDT sample</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>unmatched</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>No matching analyzed antibody or chain found for imported structure row</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ab_HydroPatch</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>VHVL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>VH,VL</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IgFold</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Ab_HydroPatch_VHVL.pdb</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>81</v>
+      </c>
+      <c r="H5" t="n">
+        <v>78</v>
+      </c>
+      <c r="I5" t="n">
+        <v>79</v>
+      </c>
+      <c r="J5" t="n">
+        <v>77</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>High hydrophobic patch score sample</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>unmatched</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>No matching analyzed antibody or chain found for imported structure row</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ab_FAIL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ab_FAIL_failed_model.pdb</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>62</v>
+      </c>
+      <c r="H6" t="n">
+        <v>68</v>
+      </c>
+      <c r="I6" t="n">
+        <v>69</v>
+      </c>
+      <c r="J6" t="n">
+        <v>58</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Failed structure status sample</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>unmatched</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>No matching analyzed antibody or chain found for imported structure row</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>antibody_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>structure_available</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>structure_tools</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>structure_model_files</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>structure_status_summary</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>mean_plddt_min</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>mean_plddt_mean</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cdr1_plddt_min</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>cdr2_plddt_min</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>cdr3_plddt_min</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>low_confidence_cdr_count</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>high_hydrophobic_patch_flag</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>high_aggregation_patch_flag</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>high_charge_patch_flag</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>structural_risk_score</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>structural_risk_class</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>structural_review_reason</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>structural_next_step_recommendation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ab001</t>
+        </is>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IgFold</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ab001_VHVL.pdb</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PASS (1)</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>86</v>
+      </c>
+      <c r="I2" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>82</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>No major structural risk flag detected from imported metrics</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Imported structure metrics do not indicate a major structural review flag in this MVP assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BsAb001</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BsAb001_ArmA_model.pdb</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>WARNING (1)</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>76</v>
+      </c>
+      <c r="G3" t="n">
+        <v>76</v>
+      </c>
+      <c r="H3" t="n">
+        <v>74</v>
+      </c>
+      <c r="I3" t="n">
+        <v>72</v>
+      </c>
+      <c r="J3" t="n">
+        <v>71</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>3</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>No major structural risk flag detected from imported metrics</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Review imported structure confidence and patch annotations before progression</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BadSeq001</t>
+        </is>
+      </c>
+      <c r="B4" t="b">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>No external structure prediction result was provided</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Import external structure prediction summary metrics if structural triage is needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Full001</t>
+        </is>
+      </c>
+      <c r="B5" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>No external structure prediction result was provided</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Import external structure prediction summary metrics if structural triage is needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VHH001</t>
+        </is>
+      </c>
+      <c r="B6" t="b">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>No external structure prediction result was provided</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Import external structure prediction summary metrics if structural triage is needed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5699,7 +6749,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -5770,7 +6820,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -5841,7 +6891,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -5912,7 +6962,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -5983,7 +7033,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -6054,7 +7104,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -6125,7 +7175,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -6196,7 +7246,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>IMGT numbering failed: No module named 'anarci'</t>
+          <t>AbNumber/ANARCI is not available: No module named 'abnumber'</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">

</xml_diff>